<commit_message>
dados do painel — 01/09 10:49
</commit_message>
<xml_diff>
--- a/data/categorias.xlsx
+++ b/data/categorias.xlsx
@@ -654,7 +654,7 @@
         <v>144677.3</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>30.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="6">
@@ -714,7 +714,7 @@
         <v>163976.29</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>28.3</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="8">
@@ -7388,7 +7388,7 @@
         <v>-35.1</v>
       </c>
       <c r="J160" s="4" t="n">
-        <v>38.5</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="161">
@@ -7540,7 +7540,7 @@
         <v>14.8</v>
       </c>
       <c r="J164" s="4" t="n">
-        <v>32.9</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="165">
@@ -11796,7 +11796,7 @@
         <v>6.4</v>
       </c>
       <c r="J276" s="4" t="n">
-        <v>16.8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="277">

</xml_diff>

<commit_message>
dados do painel — 01/09 12:12
</commit_message>
<xml_diff>
--- a/data/categorias.xlsx
+++ b/data/categorias.xlsx
@@ -684,7 +684,7 @@
         <v>136117.83</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>27</v>
+        <v>27.2</v>
       </c>
     </row>
     <row r="7">
@@ -744,7 +744,7 @@
         <v>263968.8</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="9">
@@ -9630,7 +9630,7 @@
         <v>-73.5</v>
       </c>
       <c r="J219" s="7" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="220">
@@ -11872,7 +11872,7 @@
         <v>-24.1</v>
       </c>
       <c r="J278" s="4" t="n">
-        <v>37.9</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="279">
@@ -12176,7 +12176,7 @@
         <v>16.1</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>28.7</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="287">
@@ -14024,7 +14024,7 @@
         <v>-16.9</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>28.4</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="3">
@@ -14214,7 +14214,7 @@
         <v>13.2</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>21.2</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="8">
@@ -14366,7 +14366,7 @@
         <v>-53.3</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>8.1</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="12">
@@ -14404,7 +14404,7 @@
         <v>-31.2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>20</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="13">
@@ -14518,7 +14518,7 @@
         <v>-19.4</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>-3</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="16">
@@ -14898,7 +14898,7 @@
         <v>-33.1</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>11.8</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="26">
@@ -15012,7 +15012,7 @@
         <v>13.8</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>10.1</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
dados do painel — 08/09 11:47
</commit_message>
<xml_diff>
--- a/data/categorias.xlsx
+++ b/data/categorias.xlsx
@@ -564,7 +564,7 @@
         <v>202488.42</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>33.5</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="3">
@@ -594,7 +594,7 @@
         <v>71162.42999999999</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>30.8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -654,7 +654,7 @@
         <v>131427.26</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>32.1</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="6">
@@ -714,7 +714,7 @@
         <v>148739.06</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>30.5</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="8">
@@ -834,7 +834,7 @@
         <v>190202.65</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="12">
@@ -894,7 +894,7 @@
         <v>186995.25</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="14">
@@ -1574,7 +1574,7 @@
         <v>75.2</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>26.3</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="8">
@@ -1992,7 +1992,7 @@
         <v>48.8</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>13.4</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="19">
@@ -2372,7 +2372,7 @@
         <v>-18.4</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>49.9</v>
+        <v>24.9</v>
       </c>
     </row>
     <row r="29">
@@ -2676,7 +2676,7 @@
         <v>100</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>43.5</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="37">
@@ -3056,7 +3056,7 @@
         <v>0.3</v>
       </c>
       <c r="J46" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="47">
@@ -4462,7 +4462,7 @@
         <v>-33.4</v>
       </c>
       <c r="J83" s="7" t="n">
-        <v>27.2</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="84">
@@ -7084,7 +7084,7 @@
         <v>-7.6</v>
       </c>
       <c r="J152" s="4" t="n">
-        <v>29.3</v>
+        <v>43.6</v>
       </c>
     </row>
     <row r="153">
@@ -7122,7 +7122,7 @@
         <v>9.5</v>
       </c>
       <c r="J153" s="7" t="n">
-        <v>26.3</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="154">
@@ -7312,7 +7312,7 @@
         <v>-23.9</v>
       </c>
       <c r="J158" s="4" t="n">
-        <v>36.7</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="159">
@@ -8756,7 +8756,7 @@
         <v>-13.6</v>
       </c>
       <c r="J196" s="4" t="n">
-        <v>40.6</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="197">
@@ -9022,7 +9022,7 @@
         <v>-9.800000000000001</v>
       </c>
       <c r="J203" s="7" t="n">
-        <v>20</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="204">
@@ -11834,7 +11834,7 @@
         <v>-20.2</v>
       </c>
       <c r="J277" s="7" t="n">
-        <v>27.2</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="278">
@@ -16760,7 +16760,7 @@
         <v>-1.4</v>
       </c>
       <c r="J82" s="4" t="n">
-        <v>25.5</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="83">
@@ -17178,7 +17178,7 @@
         <v>-3.2</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="94">
@@ -17330,7 +17330,7 @@
         <v>2.2</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>11.3</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="98">
@@ -17672,7 +17672,7 @@
         <v>-63.7</v>
       </c>
       <c r="J106" s="4" t="n">
-        <v>1.2</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="107">
@@ -19382,7 +19382,7 @@
         <v>-36</v>
       </c>
       <c r="J151" s="7" t="n">
-        <v>25.9</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="152">

</xml_diff>